<commit_message>
Remove isManager from emloyees
</commit_message>
<xml_diff>
--- a/src/renderer/public/template.xlsx
+++ b/src/renderer/public/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akito\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2E4FC59-BBF0-4DC9-8D83-54070B15892A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3105D35E-DDF1-4D55-8C2F-C5D6A5FC19B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>firstName</t>
   </si>
@@ -41,9 +41,6 @@
   </si>
   <si>
     <t>affiliation</t>
-  </si>
-  <si>
-    <t>isManager</t>
   </si>
   <si>
     <t>lastPromotionDate</t>
@@ -460,13 +457,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="19" width="15.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="14.4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="14.4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -521,34 +518,35 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
     </row>
-    <row r="2" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="8" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="9" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="10" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
-    <row r="16" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="15" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:18" ht="14.4" x14ac:dyDescent="0.2"/>
     <row r="17" ht="14.4" x14ac:dyDescent="0.2"/>
     <row r="18" ht="14.4" x14ac:dyDescent="0.2"/>
     <row r="19" ht="14.4" x14ac:dyDescent="0.2"/>
     <row r="20" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="21" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="22" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="23" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="24" ht="14.4" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:S1 A20:I20 A2:I19" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:R1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix import employee feature
</commit_message>
<xml_diff>
--- a/src/renderer/public/template.xlsx
+++ b/src/renderer/public/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akito\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27EFF8A-12CA-406E-A16F-52A25A25701F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5602347E-3727-4687-8675-2397B8BEF7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>firstName</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>position</t>
-  </si>
-  <si>
-    <t>baseSalary</t>
   </si>
   <si>
     <t>affiliation</t>
@@ -119,8 +116,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -460,13 +458,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="19" width="15.796875" customWidth="1"/>
+    <col min="1" max="18" width="15.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="14.4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -521,16 +519,16 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
     </row>
-    <row r="2" spans="1:19" ht="14.4" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="D2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:S1 K2:S2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F1 J2:R2 G1:R1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>